<commit_message>
Correct the commercial building retrofit cost inputs (BRESaC) against PNNL's Advanced Energy Retrofit Guide for offices: use the boiler replacement measure (HW15) that PNNL puts in the deep retrofit package instead of the burner measure (HW16) whose costs and savings had been entered under its name; count the upgrade from pneumatic to digital zone controls once rather than in four measures (its cost is HA14 minus HA12); fix two cost typos (HW8 Hot & Dry 45,190; HA14 Hot & Dry 228,927); and replace the climate totals' drifting ranges, which had left roof insulation out of the Marine zone. Commercial retrofit cost falls from 0.000241 to 0.000163 $/BTU saved and savings rise from 58.8% to 64.0% of heating and cooling energy. SoBRCbIC's commercial row is rebuilt from the corrected measures. Default results are unchanged; under a 20% retrofit policy, commercial retrofit spending is 26% lower and 2050 CO2e is 1.9 Mt lower.
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/InputData/bldgs/SoBRCbIC/Shr of Bldg Retrofitting Costs by ISIC Code.xlsx
+++ b/InputData/bldgs/SoBRCbIC/Shr of Bldg Retrofitting Costs by ISIC Code.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\DanOBrien\Models\EPS\US\eps-us\.claude\worktrees\retrofit-isic-split\InputData\bldgs\SoBRCbIC\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{00A1607B-485C-4F41-8217-525137EB6038}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{11FF655D-55BE-4444-9815-051229B28EE4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -44,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1314" uniqueCount="447">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1317" uniqueCount="450">
   <si>
     <t>SoBRCbIC Shr of Bldg Retrofitting Costs by ISIC Code</t>
   </si>
@@ -214,7 +214,7 @@
     <t>Commercial</t>
   </si>
   <si>
-    <t>For each measure BRESaC counts, PNNL gives an equipment cost and an installation cost in five climate zones. Each climate zone is weighted by its share of BRESaC's average cost per BTU (floorspace times cost per BTU), and within a zone each measure by its share of that zone's cost. Commercial heating and cooling get the same split, because the measures serve both.</t>
+    <t>For each measure BRESaC counts, PNNL gives an equipment cost and an installation cost in five climate zones. Each climate zone is weighted by its share of BRESaC's average cost per BTU (floorspace times cost per BTU), and within a zone each measure by its share of that zone's cost. Commercial heating and cooling get the same split, because the measures serve both. PNNL prices four of the measures (HA13, HA14, HA15 and HW15) as if each one had to upgrade the building's zone controls from pneumatic to digital. A building only does that once, so it is counted once, in HA13, as BRESaC does; the upgrade's cost is HA14 minus HA12, two versions of the same measure with and without it.</t>
   </si>
   <si>
     <t>What is not covered</t>
@@ -995,7 +995,7 @@
     <t>HW12 Add a VFD to One Chiller</t>
   </si>
   <si>
-    <t>HW15 Replace Boiler Burners with Modulating Burners</t>
+    <t>HW15 Replace Boilers and Change Heating Plant Pumping System to Variable Flow Primary</t>
   </si>
   <si>
     <t>A. Residential: how much of retrofit spending is envelope work</t>
@@ -1147,6 +1147,19 @@
     <t>Total cost of the counted measures in one building ($)</t>
   </si>
   <si>
+    <t>Digital zone control upgrade
+equipment ($)
+HA14 minus HA12</t>
+  </si>
+  <si>
+    <t>Digital zone control upgrade
+installation ($)
+HA14 minus HA12</t>
+  </si>
+  <si>
+    <t>HA13, HA14, HA15 and HW15 each include the full upgrade from pneumatic to digital zone controls. It is counted once, in HA13; the other three have it subtracted.</t>
+  </si>
+  <si>
     <t>BRESaC measure</t>
   </si>
   <si>
@@ -1276,7 +1289,7 @@
     <t>VFD for one chiller compressor</t>
   </si>
   <si>
-    <t>Modulating boiler burners</t>
+    <t>Condensing boilers and pumps (DDC upgrade counted under HA13)</t>
   </si>
   <si>
     <t>Total cost of counted measures in one building ($)</t>
@@ -2096,7 +2109,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="44" spans="1:2" ht="60" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:2" ht="90" x14ac:dyDescent="0.25">
       <c r="A44" s="5" t="s">
         <v>55</v>
       </c>
@@ -5287,19 +5300,19 @@
       </c>
       <c r="V2">
         <f>INDEX(Calcs!$F$58:$F$109,MATCH(V$1,Calcs!$A$58:$A$109,0))</f>
-        <v>0</v>
+        <v>6.2652119642991694E-2</v>
       </c>
       <c r="W2">
         <f>INDEX(Calcs!$F$58:$F$109,MATCH(W$1,Calcs!$A$58:$A$109,0))</f>
-        <v>0.15189975434567671</v>
+        <v>8.2476824567215584E-2</v>
       </c>
       <c r="X2">
         <f>INDEX(Calcs!$F$58:$F$109,MATCH(X$1,Calcs!$A$58:$A$109,0))</f>
-        <v>2.4713665761134956E-2</v>
+        <v>3.5622900571994909E-2</v>
       </c>
       <c r="Y2">
         <f>INDEX(Calcs!$F$58:$F$109,MATCH(Y$1,Calcs!$A$58:$A$109,0))</f>
-        <v>6.7850177477708955E-3</v>
+        <v>7.446325552416035E-3</v>
       </c>
       <c r="Z2">
         <f>INDEX(Calcs!$F$58:$F$109,MATCH(Z$1,Calcs!$A$58:$A$109,0))</f>
@@ -5331,15 +5344,15 @@
       </c>
       <c r="AG2">
         <f>INDEX(Calcs!$F$58:$F$109,MATCH(AG$1,Calcs!$A$58:$A$109,0))</f>
-        <v>0.75594162438251167</v>
+        <v>0.70452348304815571</v>
       </c>
       <c r="AH2">
         <f>INDEX(Calcs!$F$58:$F$109,MATCH(AH$1,Calcs!$A$58:$A$109,0))</f>
-        <v>5.5813720451677588E-2</v>
+        <v>0.10240893888644097</v>
       </c>
       <c r="AI2">
         <f>INDEX(Calcs!$F$58:$F$109,MATCH(AI$1,Calcs!$A$58:$A$109,0))</f>
-        <v>4.8462173112280597E-3</v>
+        <v>4.8694077307852874E-3</v>
       </c>
       <c r="AJ2">
         <f>INDEX(Calcs!$F$58:$F$109,MATCH(AJ$1,Calcs!$A$58:$A$109,0))</f>
@@ -5500,19 +5513,19 @@
       </c>
       <c r="V3">
         <f>INDEX(Calcs!$G$58:$G$109,MATCH(V$1,Calcs!$A$58:$A$109,0))</f>
-        <v>0</v>
+        <v>6.2652119642991694E-2</v>
       </c>
       <c r="W3">
         <f>INDEX(Calcs!$G$58:$G$109,MATCH(W$1,Calcs!$A$58:$A$109,0))</f>
-        <v>0.15189975434567671</v>
+        <v>8.2476824567215584E-2</v>
       </c>
       <c r="X3">
         <f>INDEX(Calcs!$G$58:$G$109,MATCH(X$1,Calcs!$A$58:$A$109,0))</f>
-        <v>2.4713665761134956E-2</v>
+        <v>3.5622900571994909E-2</v>
       </c>
       <c r="Y3">
         <f>INDEX(Calcs!$G$58:$G$109,MATCH(Y$1,Calcs!$A$58:$A$109,0))</f>
-        <v>6.7850177477708955E-3</v>
+        <v>7.446325552416035E-3</v>
       </c>
       <c r="Z3">
         <f>INDEX(Calcs!$G$58:$G$109,MATCH(Z$1,Calcs!$A$58:$A$109,0))</f>
@@ -5544,15 +5557,15 @@
       </c>
       <c r="AG3">
         <f>INDEX(Calcs!$G$58:$G$109,MATCH(AG$1,Calcs!$A$58:$A$109,0))</f>
-        <v>0.75594162438251167</v>
+        <v>0.70452348304815571</v>
       </c>
       <c r="AH3">
         <f>INDEX(Calcs!$G$58:$G$109,MATCH(AH$1,Calcs!$A$58:$A$109,0))</f>
-        <v>5.5813720451677588E-2</v>
+        <v>0.10240893888644097</v>
       </c>
       <c r="AI3">
         <f>INDEX(Calcs!$G$58:$G$109,MATCH(AI$1,Calcs!$A$58:$A$109,0))</f>
-        <v>4.8462173112280597E-3</v>
+        <v>4.8694077307852874E-3</v>
       </c>
       <c r="AJ3">
         <f>INDEX(Calcs!$G$58:$G$109,MATCH(AJ$1,Calcs!$A$58:$A$109,0))</f>
@@ -14816,7 +14829,7 @@
         <v>0.40566317524959927</v>
       </c>
       <c r="C37">
-        <v>1.650456547179108E-4</v>
+        <v>9.1827574525745243E-5</v>
       </c>
     </row>
     <row r="38" spans="1:4" x14ac:dyDescent="0.25">
@@ -14827,7 +14840,7 @@
         <v>6.1563024941687562E-2</v>
       </c>
       <c r="C38">
-        <v>2.6529571746559228E-4</v>
+        <v>1.959678809919428E-4</v>
       </c>
     </row>
     <row r="39" spans="1:4" x14ac:dyDescent="0.25">
@@ -14838,7 +14851,7 @@
         <v>3.7672564038317383E-2</v>
       </c>
       <c r="C39">
-        <v>2.00824058530716E-4</v>
+        <v>1.9606404513407841E-4</v>
       </c>
     </row>
     <row r="40" spans="1:4" x14ac:dyDescent="0.25">
@@ -14849,7 +14862,7 @@
         <v>0.45140543049506737</v>
       </c>
       <c r="C40">
-        <v>3.021342683414829E-4</v>
+        <v>2.1417364549585339E-4</v>
       </c>
     </row>
     <row r="41" spans="1:4" x14ac:dyDescent="0.25">
@@ -14860,7 +14873,7 @@
         <v>4.3695805275328507E-2</v>
       </c>
       <c r="C41">
-        <v>3.1782992160278752E-4</v>
+        <v>2.152723271593618E-4</v>
       </c>
     </row>
     <row r="43" spans="1:4" x14ac:dyDescent="0.25">
@@ -16306,6 +16319,12 @@
       <c r="E31" s="6" t="s">
         <v>362</v>
       </c>
+      <c r="F31" s="6" t="s">
+        <v>363</v>
+      </c>
+      <c r="G31" s="6" t="s">
+        <v>364</v>
+      </c>
     </row>
     <row r="32" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
@@ -16317,15 +16336,23 @@
       </c>
       <c r="C32" s="15">
         <f>'EPS Inputs'!C37</f>
-        <v>1.650456547179108E-4</v>
+        <v>9.1827574525745243E-5</v>
       </c>
       <c r="D32" s="13">
         <f>B32*C32/SUMPRODUCT($B$32:$B$36,$C$32:$C$36)</f>
-        <v>0.27767041869010334</v>
+        <v>0.22883272058703505</v>
       </c>
       <c r="E32" s="7">
         <f>G51</f>
-        <v>857499</v>
+        <v>477093</v>
+      </c>
+      <c r="F32" s="7">
+        <f>SUMIFS('PNNL Office Measures'!$E$5:$E$69,'PNNL Office Measures'!$A$5:$A$69,"HA14",'PNNL Office Measures'!$D$5:$D$69,$A32)-SUMIFS('PNNL Office Measures'!$E$5:$E$69,'PNNL Office Measures'!$A$5:$A$69,"HA12",'PNNL Office Measures'!$D$5:$D$69,$A32)</f>
+        <v>61907</v>
+      </c>
+      <c r="G32" s="7">
+        <f>SUMIFS('PNNL Office Measures'!$F$5:$F$69,'PNNL Office Measures'!$A$5:$A$69,"HA14",'PNNL Office Measures'!$D$5:$D$69,$A32)-SUMIFS('PNNL Office Measures'!$F$5:$F$69,'PNNL Office Measures'!$A$5:$A$69,"HA12",'PNNL Office Measures'!$D$5:$D$69,$A32)</f>
+        <v>128296</v>
       </c>
     </row>
     <row r="33" spans="1:28" x14ac:dyDescent="0.25">
@@ -16338,15 +16365,23 @@
       </c>
       <c r="C33" s="15">
         <f>'EPS Inputs'!C38</f>
-        <v>2.6529571746559228E-4</v>
+        <v>1.959678809919428E-4</v>
       </c>
       <c r="D33" s="13">
         <f>B33*C33/SUMPRODUCT($B$32:$B$36,$C$32:$C$36)</f>
-        <v>6.7734530541031013E-2</v>
+        <v>7.4111272907158104E-2</v>
       </c>
       <c r="E33" s="7">
         <f>J51</f>
-        <v>1383954</v>
+        <v>1000130</v>
+      </c>
+      <c r="F33" s="7">
+        <f>SUMIFS('PNNL Office Measures'!$E$5:$E$69,'PNNL Office Measures'!$A$5:$A$69,"HA14",'PNNL Office Measures'!$D$5:$D$69,$A33)-SUMIFS('PNNL Office Measures'!$E$5:$E$69,'PNNL Office Measures'!$A$5:$A$69,"HA12",'PNNL Office Measures'!$D$5:$D$69,$A33)</f>
+        <v>62463</v>
+      </c>
+      <c r="G33" s="7">
+        <f>SUMIFS('PNNL Office Measures'!$F$5:$F$69,'PNNL Office Measures'!$A$5:$A$69,"HA14",'PNNL Office Measures'!$D$5:$D$69,$A33)-SUMIFS('PNNL Office Measures'!$F$5:$F$69,'PNNL Office Measures'!$A$5:$A$69,"HA12",'PNNL Office Measures'!$D$5:$D$69,$A33)</f>
+        <v>129449</v>
       </c>
     </row>
     <row r="34" spans="1:28" x14ac:dyDescent="0.25">
@@ -16359,15 +16394,23 @@
       </c>
       <c r="C34" s="15">
         <f>'EPS Inputs'!C39</f>
-        <v>2.00824058530716E-4</v>
+        <v>1.9606404513407841E-4</v>
       </c>
       <c r="D34" s="13">
         <f>B34*C34/SUMPRODUCT($B$32:$B$36,$C$32:$C$36)</f>
-        <v>3.1376236805193393E-2</v>
+        <v>4.5373529505810681E-2</v>
       </c>
       <c r="E34" s="7">
         <f>M51</f>
-        <v>1217854</v>
+        <v>1018935</v>
+      </c>
+      <c r="F34" s="7">
+        <f>SUMIFS('PNNL Office Measures'!$E$5:$E$69,'PNNL Office Measures'!$A$5:$A$69,"HA14",'PNNL Office Measures'!$D$5:$D$69,$A34)-SUMIFS('PNNL Office Measures'!$E$5:$E$69,'PNNL Office Measures'!$A$5:$A$69,"HA12",'PNNL Office Measures'!$D$5:$D$69,$A34)</f>
+        <v>64690</v>
+      </c>
+      <c r="G34" s="7">
+        <f>SUMIFS('PNNL Office Measures'!$F$5:$F$69,'PNNL Office Measures'!$A$5:$A$69,"HA14",'PNNL Office Measures'!$D$5:$D$69,$A34)-SUMIFS('PNNL Office Measures'!$F$5:$F$69,'PNNL Office Measures'!$A$5:$A$69,"HA12",'PNNL Office Measures'!$D$5:$D$69,$A34)</f>
+        <v>134064</v>
       </c>
     </row>
     <row r="35" spans="1:28" x14ac:dyDescent="0.25">
@@ -16380,15 +16423,23 @@
       </c>
       <c r="C35" s="15">
         <f>'EPS Inputs'!C40</f>
-        <v>3.021342683414829E-4</v>
+        <v>2.1417364549585339E-4</v>
       </c>
       <c r="D35" s="13">
         <f>B35*C35/SUMPRODUCT($B$32:$B$36,$C$32:$C$36)</f>
-        <v>0.56562253018493103</v>
+        <v>0.59389850677350708</v>
       </c>
       <c r="E35" s="7">
         <f>P51</f>
-        <v>1238255</v>
+        <v>1051099</v>
+      </c>
+      <c r="F35" s="7">
+        <f>SUMIFS('PNNL Office Measures'!$E$5:$E$69,'PNNL Office Measures'!$A$5:$A$69,"HA14",'PNNL Office Measures'!$D$5:$D$69,$A35)-SUMIFS('PNNL Office Measures'!$E$5:$E$69,'PNNL Office Measures'!$A$5:$A$69,"HA12",'PNNL Office Measures'!$D$5:$D$69,$A35)</f>
+        <v>61226</v>
+      </c>
+      <c r="G35" s="7">
+        <f>SUMIFS('PNNL Office Measures'!$F$5:$F$69,'PNNL Office Measures'!$A$5:$A$69,"HA14",'PNNL Office Measures'!$D$5:$D$69,$A35)-SUMIFS('PNNL Office Measures'!$F$5:$F$69,'PNNL Office Measures'!$A$5:$A$69,"HA12",'PNNL Office Measures'!$D$5:$D$69,$A35)</f>
+        <v>126886</v>
       </c>
     </row>
     <row r="36" spans="1:28" x14ac:dyDescent="0.25">
@@ -16401,101 +16452,114 @@
       </c>
       <c r="C36" s="15">
         <f>'EPS Inputs'!C41</f>
-        <v>3.1782992160278752E-4</v>
+        <v>2.152723271593618E-4</v>
       </c>
       <c r="D36" s="13">
         <f>B36*C36/SUMPRODUCT($B$32:$B$36,$C$32:$C$36)</f>
-        <v>5.7596283778741306E-2</v>
+        <v>5.7783970226489186E-2</v>
       </c>
       <c r="E36" s="7">
         <f>S51</f>
-        <v>1225958</v>
+        <v>1056492</v>
+      </c>
+      <c r="F36" s="7">
+        <f>SUMIFS('PNNL Office Measures'!$E$5:$E$69,'PNNL Office Measures'!$A$5:$A$69,"HA14",'PNNL Office Measures'!$D$5:$D$69,$A36)-SUMIFS('PNNL Office Measures'!$E$5:$E$69,'PNNL Office Measures'!$A$5:$A$69,"HA12",'PNNL Office Measures'!$D$5:$D$69,$A36)</f>
+        <v>60979</v>
+      </c>
+      <c r="G36" s="7">
+        <f>SUMIFS('PNNL Office Measures'!$F$5:$F$69,'PNNL Office Measures'!$A$5:$A$69,"HA14",'PNNL Office Measures'!$D$5:$D$69,$A36)-SUMIFS('PNNL Office Measures'!$F$5:$F$69,'PNNL Office Measures'!$A$5:$A$69,"HA12",'PNNL Office Measures'!$D$5:$D$69,$A36)</f>
+        <v>126374</v>
+      </c>
+    </row>
+    <row r="37" spans="1:28" x14ac:dyDescent="0.25">
+      <c r="A37" t="s">
+        <v>365</v>
       </c>
     </row>
     <row r="39" spans="1:28" ht="96" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A39" s="6" t="s">
-        <v>363</v>
+        <v>366</v>
       </c>
       <c r="B39" s="6" t="s">
-        <v>364</v>
+        <v>367</v>
       </c>
       <c r="C39" s="6" t="s">
-        <v>365</v>
+        <v>368</v>
       </c>
       <c r="D39" s="6" t="s">
-        <v>366</v>
+        <v>369</v>
       </c>
       <c r="E39" s="6" t="s">
-        <v>367</v>
+        <v>370</v>
       </c>
       <c r="F39" s="6" t="s">
-        <v>368</v>
+        <v>371</v>
       </c>
       <c r="G39" s="6" t="s">
-        <v>369</v>
+        <v>372</v>
       </c>
       <c r="H39" s="6" t="s">
-        <v>370</v>
+        <v>373</v>
       </c>
       <c r="I39" s="6" t="s">
-        <v>371</v>
+        <v>374</v>
       </c>
       <c r="J39" s="6" t="s">
-        <v>372</v>
+        <v>375</v>
       </c>
       <c r="K39" s="6" t="s">
-        <v>373</v>
+        <v>376</v>
       </c>
       <c r="L39" s="6" t="s">
-        <v>374</v>
+        <v>377</v>
       </c>
       <c r="M39" s="6" t="s">
-        <v>375</v>
+        <v>378</v>
       </c>
       <c r="N39" s="6" t="s">
-        <v>376</v>
+        <v>379</v>
       </c>
       <c r="O39" s="6" t="s">
-        <v>377</v>
+        <v>380</v>
       </c>
       <c r="P39" s="6" t="s">
-        <v>378</v>
+        <v>381</v>
       </c>
       <c r="Q39" s="6" t="s">
-        <v>379</v>
+        <v>382</v>
       </c>
       <c r="R39" s="6" t="s">
-        <v>380</v>
+        <v>383</v>
       </c>
       <c r="S39" s="6" t="s">
-        <v>381</v>
+        <v>384</v>
       </c>
       <c r="T39" s="6" t="s">
-        <v>382</v>
+        <v>385</v>
       </c>
       <c r="U39" s="6" t="s">
-        <v>383</v>
+        <v>386</v>
       </c>
       <c r="V39" s="6" t="s">
-        <v>384</v>
+        <v>387</v>
       </c>
       <c r="W39" s="6" t="s">
-        <v>385</v>
+        <v>388</v>
       </c>
       <c r="X39" s="6" t="s">
-        <v>386</v>
+        <v>389</v>
       </c>
       <c r="Y39" s="6" t="s">
-        <v>387</v>
+        <v>390</v>
       </c>
       <c r="Z39" s="6" t="s">
-        <v>388</v>
+        <v>391</v>
       </c>
       <c r="AA39" s="6" t="s">
-        <v>389</v>
+        <v>392</v>
       </c>
       <c r="AB39" s="6" t="s">
-        <v>390</v>
+        <v>393</v>
       </c>
     </row>
     <row r="40" spans="1:28" x14ac:dyDescent="0.25">
@@ -16506,7 +16570,7 @@
         <v>116</v>
       </c>
       <c r="C40" t="s">
-        <v>391</v>
+        <v>394</v>
       </c>
       <c r="D40" t="s">
         <v>353</v>
@@ -16576,11 +16640,11 @@
       </c>
       <c r="U40" s="13">
         <f t="shared" ref="U40:U50" si="0">$D$32*F40*G40/$E$32+$D$33*I40*J40/$E$33+$D$34*L40*M40/$E$34+$D$35*O40*P40/$E$35+$D$36*R40*S40/$E$36</f>
-        <v>7.9945788554424455E-2</v>
+        <v>0.10207593361326465</v>
       </c>
       <c r="V40" s="13">
         <f t="shared" ref="V40:V50" si="1">$D$32*F40*H40/$E$32+$D$33*I40*K40/$E$33+$D$34*L40*N40/$E$34+$D$35*O40*Q40/$E$35+$D$36*R40*T40/$E$36</f>
-        <v>0.1365406317534561</v>
+        <v>0.17434078473781875</v>
       </c>
       <c r="W40" s="13">
         <f>VLOOKUP($D40,Calcs!$A$21:$J$27,8,FALSE)</f>
@@ -16596,7 +16660,7 @@
       </c>
       <c r="Z40" s="13">
         <f t="shared" ref="Z40:Z50" si="2">U40*W40</f>
-        <v>7.9945788554424455E-2</v>
+        <v>0.10207593361326465</v>
       </c>
       <c r="AA40" s="13">
         <f t="shared" ref="AA40:AA50" si="3">U40*Y40</f>
@@ -16615,7 +16679,7 @@
         <v>125</v>
       </c>
       <c r="C41" t="s">
-        <v>392</v>
+        <v>395</v>
       </c>
       <c r="D41" t="s">
         <v>345</v>
@@ -16685,11 +16749,11 @@
       </c>
       <c r="U41" s="13">
         <f t="shared" si="0"/>
-        <v>5.9727962067220614E-2</v>
+        <v>8.0706420718736266E-2</v>
       </c>
       <c r="V41" s="13">
         <f t="shared" si="1"/>
-        <v>0.13230684822690952</v>
+        <v>0.17877742221801018</v>
       </c>
       <c r="W41" s="13">
         <f>VLOOKUP($D41,Calcs!$A$21:$J$27,8,FALSE)</f>
@@ -16705,15 +16769,15 @@
       </c>
       <c r="Z41" s="13">
         <f t="shared" si="2"/>
-        <v>4.8801656663865704E-2</v>
+        <v>6.5942431286247036E-2</v>
       </c>
       <c r="AA41" s="13">
         <f t="shared" si="3"/>
-        <v>9.5158528986189015E-3</v>
+        <v>1.285813881727977E-2</v>
       </c>
       <c r="AB41" s="13">
         <f t="shared" si="4"/>
-        <v>1.4104525047360032E-3</v>
+        <v>1.9058506152094521E-3</v>
       </c>
     </row>
     <row r="42" spans="1:28" x14ac:dyDescent="0.25">
@@ -16724,7 +16788,7 @@
         <v>127</v>
       </c>
       <c r="C42" t="s">
-        <v>393</v>
+        <v>396</v>
       </c>
       <c r="D42" t="s">
         <v>345</v>
@@ -16737,68 +16801,68 @@
         <v>1</v>
       </c>
       <c r="G42" s="7">
-        <f>SUMIFS('PNNL Office Measures'!$E$5:$E$69,'PNNL Office Measures'!$A$5:$A$69,$B42,'PNNL Office Measures'!$D$5:$D$69,"Hot &amp; Humid")</f>
-        <v>61907</v>
+        <f>SUMIFS('PNNL Office Measures'!$E$5:$E$69,'PNNL Office Measures'!$A$5:$A$69,$B42,'PNNL Office Measures'!$D$5:$D$69,"Hot &amp; Humid")-$F$32</f>
+        <v>0</v>
       </c>
       <c r="H42" s="7">
-        <f>SUMIFS('PNNL Office Measures'!$F$5:$F$69,'PNNL Office Measures'!$A$5:$A$69,$B42,'PNNL Office Measures'!$D$5:$D$69,"Hot &amp; Humid")</f>
-        <v>164980</v>
+        <f>SUMIFS('PNNL Office Measures'!$F$5:$F$69,'PNNL Office Measures'!$A$5:$A$69,$B42,'PNNL Office Measures'!$D$5:$D$69,"Hot &amp; Humid")-$G$32</f>
+        <v>36684</v>
       </c>
       <c r="I42">
         <f>SUMIFS('EPS Inputs'!$C$45:$C$99,'EPS Inputs'!$A$45:$A$99,"Hot &amp; Dry",'EPS Inputs'!$D$45:$D$99,$A42)</f>
         <v>1</v>
       </c>
       <c r="J42" s="7">
-        <f>SUMIFS('PNNL Office Measures'!$E$5:$E$69,'PNNL Office Measures'!$A$5:$A$69,$B42,'PNNL Office Measures'!$D$5:$D$69,"Hot &amp; Dry")</f>
-        <v>62463</v>
+        <f>SUMIFS('PNNL Office Measures'!$E$5:$E$69,'PNNL Office Measures'!$A$5:$A$69,$B42,'PNNL Office Measures'!$D$5:$D$69,"Hot &amp; Dry")-$F$33</f>
+        <v>0</v>
       </c>
       <c r="K42" s="7">
-        <f>SUMIFS('PNNL Office Measures'!$F$5:$F$69,'PNNL Office Measures'!$A$5:$A$69,$B42,'PNNL Office Measures'!$D$5:$D$69,"Hot &amp; Dry")</f>
-        <v>166463</v>
+        <f>SUMIFS('PNNL Office Measures'!$F$5:$F$69,'PNNL Office Measures'!$A$5:$A$69,$B42,'PNNL Office Measures'!$D$5:$D$69,"Hot &amp; Dry")-$G$33</f>
+        <v>37014</v>
       </c>
       <c r="L42">
         <f>SUMIFS('EPS Inputs'!$C$45:$C$99,'EPS Inputs'!$A$45:$A$99,"Marine",'EPS Inputs'!$D$45:$D$99,$A42)</f>
         <v>1</v>
       </c>
       <c r="M42" s="7">
-        <f>SUMIFS('PNNL Office Measures'!$E$5:$E$69,'PNNL Office Measures'!$A$5:$A$69,$B42,'PNNL Office Measures'!$D$5:$D$69,"Marine")</f>
-        <v>64690</v>
+        <f>SUMIFS('PNNL Office Measures'!$E$5:$E$69,'PNNL Office Measures'!$A$5:$A$69,$B42,'PNNL Office Measures'!$D$5:$D$69,"Marine")-$F$34</f>
+        <v>0</v>
       </c>
       <c r="N42" s="7">
-        <f>SUMIFS('PNNL Office Measures'!$F$5:$F$69,'PNNL Office Measures'!$A$5:$A$69,$B42,'PNNL Office Measures'!$D$5:$D$69,"Marine")</f>
-        <v>172397</v>
+        <f>SUMIFS('PNNL Office Measures'!$F$5:$F$69,'PNNL Office Measures'!$A$5:$A$69,$B42,'PNNL Office Measures'!$D$5:$D$69,"Marine")-$G$34</f>
+        <v>38333</v>
       </c>
       <c r="O42">
         <f>SUMIFS('EPS Inputs'!$C$45:$C$99,'EPS Inputs'!$A$45:$A$99,"Cold",'EPS Inputs'!$D$45:$D$99,$A42)</f>
         <v>1</v>
       </c>
       <c r="P42" s="7">
-        <f>SUMIFS('PNNL Office Measures'!$E$5:$E$69,'PNNL Office Measures'!$A$5:$A$69,$B42,'PNNL Office Measures'!$D$5:$D$69,"Cold")</f>
-        <v>61226</v>
+        <f>SUMIFS('PNNL Office Measures'!$E$5:$E$69,'PNNL Office Measures'!$A$5:$A$69,$B42,'PNNL Office Measures'!$D$5:$D$69,"Cold")-$F$35</f>
+        <v>0</v>
       </c>
       <c r="Q42" s="7">
-        <f>SUMIFS('PNNL Office Measures'!$F$5:$F$69,'PNNL Office Measures'!$A$5:$A$69,$B42,'PNNL Office Measures'!$D$5:$D$69,"Cold")</f>
-        <v>163167</v>
+        <f>SUMIFS('PNNL Office Measures'!$F$5:$F$69,'PNNL Office Measures'!$A$5:$A$69,$B42,'PNNL Office Measures'!$D$5:$D$69,"Cold")-$G$35</f>
+        <v>36281</v>
       </c>
       <c r="R42">
         <f>SUMIFS('EPS Inputs'!$C$45:$C$99,'EPS Inputs'!$A$45:$A$99,"Very Cold",'EPS Inputs'!$D$45:$D$99,$A42)</f>
         <v>1</v>
       </c>
       <c r="S42" s="7">
-        <f>SUMIFS('PNNL Office Measures'!$E$5:$E$69,'PNNL Office Measures'!$A$5:$A$69,$B42,'PNNL Office Measures'!$D$5:$D$69,"Very Cold")</f>
-        <v>60979</v>
+        <f>SUMIFS('PNNL Office Measures'!$E$5:$E$69,'PNNL Office Measures'!$A$5:$A$69,$B42,'PNNL Office Measures'!$D$5:$D$69,"Very Cold")-$F$36</f>
+        <v>0</v>
       </c>
       <c r="T42" s="7">
-        <f>SUMIFS('PNNL Office Measures'!$F$5:$F$69,'PNNL Office Measures'!$A$5:$A$69,$B42,'PNNL Office Measures'!$D$5:$D$69,"Very Cold")</f>
-        <v>162508</v>
+        <f>SUMIFS('PNNL Office Measures'!$F$5:$F$69,'PNNL Office Measures'!$A$5:$A$69,$B42,'PNNL Office Measures'!$D$5:$D$69,"Very Cold")-$G$36</f>
+        <v>36134</v>
       </c>
       <c r="U42" s="13">
         <f t="shared" si="0"/>
-        <v>5.5602383932595464E-2</v>
+        <v>0</v>
       </c>
       <c r="V42" s="13">
         <f t="shared" si="1"/>
-        <v>0.14817938280020687</v>
+        <v>4.452091732574489E-2</v>
       </c>
       <c r="W42" s="13">
         <f>VLOOKUP($D42,Calcs!$A$21:$J$27,8,FALSE)</f>
@@ -16814,15 +16878,15 @@
       </c>
       <c r="Z42" s="13">
         <f t="shared" si="2"/>
-        <v>4.5430789138880739E-2</v>
+        <v>0</v>
       </c>
       <c r="AA42" s="13">
         <f t="shared" si="3"/>
-        <v>8.8585662058858015E-3</v>
+        <v>0</v>
       </c>
       <c r="AB42" s="13">
         <f t="shared" si="4"/>
-        <v>1.3130285878289231E-3</v>
+        <v>0</v>
       </c>
     </row>
     <row r="43" spans="1:28" x14ac:dyDescent="0.25">
@@ -16833,7 +16897,7 @@
         <v>129</v>
       </c>
       <c r="C43" t="s">
-        <v>394</v>
+        <v>397</v>
       </c>
       <c r="D43" t="s">
         <v>345</v>
@@ -16846,68 +16910,68 @@
         <v>1</v>
       </c>
       <c r="G43" s="7">
-        <f>SUMIFS('PNNL Office Measures'!$E$5:$E$69,'PNNL Office Measures'!$A$5:$A$69,$B43,'PNNL Office Measures'!$D$5:$D$69,"Hot &amp; Humid")</f>
-        <v>78581</v>
+        <f>SUMIFS('PNNL Office Measures'!$E$5:$E$69,'PNNL Office Measures'!$A$5:$A$69,$B43,'PNNL Office Measures'!$D$5:$D$69,"Hot &amp; Humid")-$F$32</f>
+        <v>16674</v>
       </c>
       <c r="H43" s="7">
-        <f>SUMIFS('PNNL Office Measures'!$F$5:$F$69,'PNNL Office Measures'!$A$5:$A$69,$B43,'PNNL Office Measures'!$D$5:$D$69,"Hot &amp; Humid")</f>
-        <v>154455</v>
+        <f>SUMIFS('PNNL Office Measures'!$F$5:$F$69,'PNNL Office Measures'!$A$5:$A$69,$B43,'PNNL Office Measures'!$D$5:$D$69,"Hot &amp; Humid")-$G$32</f>
+        <v>26159</v>
       </c>
       <c r="I43">
         <f>SUMIFS('EPS Inputs'!$C$45:$C$99,'EPS Inputs'!$A$45:$A$99,"Hot &amp; Dry",'EPS Inputs'!$D$45:$D$99,$A43)</f>
         <v>1</v>
       </c>
       <c r="J43" s="7">
-        <f>SUMIFS('PNNL Office Measures'!$E$5:$E$69,'PNNL Office Measures'!$A$5:$A$69,$B43,'PNNL Office Measures'!$D$5:$D$69,"Hot &amp; Dry")</f>
-        <v>79288</v>
+        <f>SUMIFS('PNNL Office Measures'!$E$5:$E$69,'PNNL Office Measures'!$A$5:$A$69,$B43,'PNNL Office Measures'!$D$5:$D$69,"Hot &amp; Dry")-$F$33</f>
+        <v>16825</v>
       </c>
       <c r="K43" s="7">
-        <f>SUMIFS('PNNL Office Measures'!$F$5:$F$69,'PNNL Office Measures'!$A$5:$A$69,$B43,'PNNL Office Measures'!$D$5:$D$69,"Hot &amp; Dry")</f>
-        <v>221372</v>
+        <f>SUMIFS('PNNL Office Measures'!$F$5:$F$69,'PNNL Office Measures'!$A$5:$A$69,$B43,'PNNL Office Measures'!$D$5:$D$69,"Hot &amp; Dry")-$G$33</f>
+        <v>91923</v>
       </c>
       <c r="L43">
         <f>SUMIFS('EPS Inputs'!$C$45:$C$99,'EPS Inputs'!$A$45:$A$99,"Marine",'EPS Inputs'!$D$45:$D$99,$A43)</f>
         <v>1</v>
       </c>
       <c r="M43" s="7">
-        <f>SUMIFS('PNNL Office Measures'!$E$5:$E$69,'PNNL Office Measures'!$A$5:$A$69,$B43,'PNNL Office Measures'!$D$5:$D$69,"Marine")</f>
-        <v>82114</v>
+        <f>SUMIFS('PNNL Office Measures'!$E$5:$E$69,'PNNL Office Measures'!$A$5:$A$69,$B43,'PNNL Office Measures'!$D$5:$D$69,"Marine")-$F$34</f>
+        <v>17424</v>
       </c>
       <c r="N43" s="7">
-        <f>SUMIFS('PNNL Office Measures'!$F$5:$F$69,'PNNL Office Measures'!$A$5:$A$69,$B43,'PNNL Office Measures'!$D$5:$D$69,"Marine")</f>
-        <v>203670</v>
+        <f>SUMIFS('PNNL Office Measures'!$F$5:$F$69,'PNNL Office Measures'!$A$5:$A$69,$B43,'PNNL Office Measures'!$D$5:$D$69,"Marine")-$G$34</f>
+        <v>69606</v>
       </c>
       <c r="O43">
         <f>SUMIFS('EPS Inputs'!$C$45:$C$99,'EPS Inputs'!$A$45:$A$99,"Cold",'EPS Inputs'!$D$45:$D$99,$A43)</f>
         <v>1</v>
       </c>
       <c r="P43" s="7">
-        <f>SUMIFS('PNNL Office Measures'!$E$5:$E$69,'PNNL Office Measures'!$A$5:$A$69,$B43,'PNNL Office Measures'!$D$5:$D$69,"Cold")</f>
-        <v>77717</v>
+        <f>SUMIFS('PNNL Office Measures'!$E$5:$E$69,'PNNL Office Measures'!$A$5:$A$69,$B43,'PNNL Office Measures'!$D$5:$D$69,"Cold")-$F$35</f>
+        <v>16491</v>
       </c>
       <c r="Q43" s="7">
-        <f>SUMIFS('PNNL Office Measures'!$F$5:$F$69,'PNNL Office Measures'!$A$5:$A$69,$B43,'PNNL Office Measures'!$D$5:$D$69,"Cold")</f>
-        <v>267669</v>
+        <f>SUMIFS('PNNL Office Measures'!$F$5:$F$69,'PNNL Office Measures'!$A$5:$A$69,$B43,'PNNL Office Measures'!$D$5:$D$69,"Cold")-$G$35</f>
+        <v>140783</v>
       </c>
       <c r="R43">
         <f>SUMIFS('EPS Inputs'!$C$45:$C$99,'EPS Inputs'!$A$45:$A$99,"Very Cold",'EPS Inputs'!$D$45:$D$99,$A43)</f>
         <v>1</v>
       </c>
       <c r="S43" s="7">
-        <f>SUMIFS('PNNL Office Measures'!$E$5:$E$69,'PNNL Office Measures'!$A$5:$A$69,$B43,'PNNL Office Measures'!$D$5:$D$69,"Very Cold")</f>
-        <v>77403</v>
+        <f>SUMIFS('PNNL Office Measures'!$E$5:$E$69,'PNNL Office Measures'!$A$5:$A$69,$B43,'PNNL Office Measures'!$D$5:$D$69,"Very Cold")-$F$36</f>
+        <v>16424</v>
       </c>
       <c r="T43" s="7">
-        <f>SUMIFS('PNNL Office Measures'!$F$5:$F$69,'PNNL Office Measures'!$A$5:$A$69,$B43,'PNNL Office Measures'!$D$5:$D$69,"Very Cold")</f>
-        <v>222928</v>
+        <f>SUMIFS('PNNL Office Measures'!$F$5:$F$69,'PNNL Office Measures'!$A$5:$A$69,$B43,'PNNL Office Measures'!$D$5:$D$69,"Very Cold")-$G$36</f>
+        <v>96554</v>
       </c>
       <c r="U43" s="13">
         <f t="shared" si="0"/>
-        <v>7.0578563365066072E-2</v>
+        <v>2.0236313318056302E-2</v>
       </c>
       <c r="V43" s="13">
         <f t="shared" si="1"/>
-        <v>0.19883837987652792</v>
+        <v>0.10728514843877061</v>
       </c>
       <c r="W43" s="13">
         <f>VLOOKUP($D43,Calcs!$A$21:$J$27,8,FALSE)</f>
@@ -16923,15 +16987,15 @@
       </c>
       <c r="Z43" s="13">
         <f t="shared" si="2"/>
-        <v>5.7667308542930243E-2</v>
+        <v>1.6534393280968545E-2</v>
       </c>
       <c r="AA43" s="13">
         <f t="shared" si="3"/>
-        <v>1.1244569604132063E-2</v>
+        <v>3.2240473989094739E-3</v>
       </c>
       <c r="AB43" s="13">
         <f t="shared" si="4"/>
-        <v>1.6666852180037643E-3</v>
+        <v>4.7787263817828171E-4</v>
       </c>
     </row>
     <row r="44" spans="1:28" x14ac:dyDescent="0.25">
@@ -16942,7 +17006,7 @@
         <v>131</v>
       </c>
       <c r="C44" t="s">
-        <v>395</v>
+        <v>398</v>
       </c>
       <c r="D44" t="s">
         <v>347</v>
@@ -17012,11 +17076,11 @@
       </c>
       <c r="U44" s="13">
         <f t="shared" si="0"/>
-        <v>1.8761196783431675E-2</v>
+        <v>2.566999336520593E-2</v>
       </c>
       <c r="V44" s="13">
         <f t="shared" si="1"/>
-        <v>1.3614427035684652E-2</v>
+        <v>1.8719483695534223E-2</v>
       </c>
       <c r="W44" s="13">
         <f>VLOOKUP($D44,Calcs!$A$21:$J$27,8,FALSE)</f>
@@ -17032,15 +17096,15 @@
       </c>
       <c r="Z44" s="13">
         <f t="shared" si="2"/>
-        <v>9.5056730369387152E-3</v>
+        <v>1.3006129971704338E-2</v>
       </c>
       <c r="AA44" s="13">
         <f t="shared" si="3"/>
-        <v>9.1572508109606984E-3</v>
+        <v>1.2529401523493371E-2</v>
       </c>
       <c r="AB44" s="13">
         <f t="shared" si="4"/>
-        <v>9.8272935532261153E-5</v>
+        <v>1.3446187000822152E-4</v>
       </c>
     </row>
     <row r="45" spans="1:28" x14ac:dyDescent="0.25">
@@ -17051,7 +17115,7 @@
         <v>133</v>
       </c>
       <c r="C45" t="s">
-        <v>396</v>
+        <v>399</v>
       </c>
       <c r="D45" t="s">
         <v>355</v>
@@ -17125,7 +17189,7 @@
       </c>
       <c r="V45" s="13">
         <f t="shared" si="1"/>
-        <v>6.8558670660983452E-4</v>
+        <v>1.0184824810839967E-3</v>
       </c>
       <c r="W45" s="13">
         <f>VLOOKUP($D45,Calcs!$A$21:$J$27,8,FALSE)</f>
@@ -17160,7 +17224,7 @@
         <v>135</v>
       </c>
       <c r="C46" t="s">
-        <v>397</v>
+        <v>400</v>
       </c>
       <c r="D46" t="s">
         <v>347</v>
@@ -17230,11 +17294,11 @@
       </c>
       <c r="U46" s="13">
         <f t="shared" si="0"/>
-        <v>1.3213566748221078E-3</v>
+        <v>2.0005960684585547E-3</v>
       </c>
       <c r="V46" s="13">
         <f t="shared" si="1"/>
-        <v>8.9036671710362937E-4</v>
+        <v>1.3480570293132096E-3</v>
       </c>
       <c r="W46" s="13">
         <f>VLOOKUP($D46,Calcs!$A$21:$J$27,8,FALSE)</f>
@@ -17250,15 +17314,15 @@
       </c>
       <c r="Z46" s="13">
         <f t="shared" si="2"/>
-        <v>6.6948738190986796E-4</v>
+        <v>1.0136353413523346E-3</v>
       </c>
       <c r="AA46" s="13">
         <f t="shared" si="3"/>
-        <v>6.4494790080602883E-4</v>
+        <v>9.7648141436667548E-4</v>
       </c>
       <c r="AB46" s="13">
         <f t="shared" si="4"/>
-        <v>6.9213921062110402E-6</v>
+        <v>1.0479312739544809E-5</v>
       </c>
     </row>
     <row r="47" spans="1:28" x14ac:dyDescent="0.25">
@@ -17269,7 +17333,7 @@
         <v>137</v>
       </c>
       <c r="C47" t="s">
-        <v>398</v>
+        <v>401</v>
       </c>
       <c r="D47" t="s">
         <v>349</v>
@@ -17339,11 +17403,11 @@
       </c>
       <c r="U47" s="13">
         <f t="shared" si="0"/>
-        <v>6.1140814711311137E-3</v>
+        <v>9.0836570373325973E-3</v>
       </c>
       <c r="V47" s="13">
         <f t="shared" si="1"/>
-        <v>3.3719072518623569E-3</v>
+        <v>5.014240597305721E-3</v>
       </c>
       <c r="W47" s="13">
         <f>VLOOKUP($D47,Calcs!$A$21:$J$27,8,FALSE)</f>
@@ -17359,15 +17423,15 @@
       </c>
       <c r="Z47" s="13">
         <f t="shared" si="2"/>
-        <v>5.0120167352119783E-3</v>
+        <v>7.446325552416035E-3</v>
       </c>
       <c r="AA47" s="13">
         <f t="shared" si="3"/>
-        <v>9.5526061537456021E-4</v>
+        <v>1.4192254146931551E-3</v>
       </c>
       <c r="AB47" s="13">
         <f t="shared" si="4"/>
-        <v>1.4680412054457527E-4</v>
+        <v>2.1810607022340695E-4</v>
       </c>
     </row>
     <row r="48" spans="1:28" x14ac:dyDescent="0.25">
@@ -17378,7 +17442,7 @@
         <v>139</v>
       </c>
       <c r="C48" t="s">
-        <v>399</v>
+        <v>402</v>
       </c>
       <c r="D48" t="s">
         <v>347</v>
@@ -17448,11 +17512,11 @@
       </c>
       <c r="U48" s="13">
         <f t="shared" si="0"/>
-        <v>1.4465896222926246E-2</v>
+        <v>2.1500409601266687E-2</v>
       </c>
       <c r="V48" s="13">
         <f t="shared" si="1"/>
-        <v>1.0636026096332674E-2</v>
+        <v>1.5817826228485501E-2</v>
       </c>
       <c r="W48" s="13">
         <f>VLOOKUP($D48,Calcs!$A$21:$J$27,8,FALSE)</f>
@@ -17468,15 +17532,15 @@
       </c>
       <c r="Z48" s="13">
         <f t="shared" si="2"/>
-        <v>7.3293874196159649E-3</v>
+        <v>1.0893540864641789E-2</v>
       </c>
       <c r="AA48" s="13">
         <f t="shared" si="3"/>
-        <v>7.0607350611901912E-3</v>
+        <v>1.0494247543475407E-2</v>
       </c>
       <c r="AB48" s="13">
         <f t="shared" si="4"/>
-        <v>7.5773742120089862E-5</v>
+        <v>1.1262119314949217E-4</v>
       </c>
     </row>
     <row r="49" spans="1:28" x14ac:dyDescent="0.25">
@@ -17487,7 +17551,7 @@
         <v>141</v>
       </c>
       <c r="C49" t="s">
-        <v>400</v>
+        <v>403</v>
       </c>
       <c r="D49" t="s">
         <v>347</v>
@@ -17557,11 +17621,11 @@
       </c>
       <c r="U49" s="13">
         <f t="shared" si="0"/>
-        <v>1.4228522215796853E-2</v>
+        <v>2.113735735716404E-2</v>
       </c>
       <c r="V49" s="13">
         <f t="shared" si="1"/>
-        <v>4.648404636395851E-3</v>
+        <v>6.9124751868122093E-3</v>
       </c>
       <c r="W49" s="13">
         <f>VLOOKUP($D49,Calcs!$A$21:$J$27,8,FALSE)</f>
@@ -17577,15 +17641,15 @@
       </c>
       <c r="Z49" s="13">
         <f t="shared" si="2"/>
-        <v>7.2091179226704064E-3</v>
+        <v>1.0709594394296447E-2</v>
       </c>
       <c r="AA49" s="13">
         <f t="shared" si="3"/>
-        <v>6.9448739386627498E-3</v>
+        <v>1.0317043471949115E-2</v>
       </c>
       <c r="AB49" s="13">
         <f t="shared" si="4"/>
-        <v>7.4530354463697794E-5</v>
+        <v>1.1071949091847831E-4</v>
       </c>
     </row>
     <row r="50" spans="1:28" x14ac:dyDescent="0.25">
@@ -17593,84 +17657,84 @@
         <v>143</v>
       </c>
       <c r="B50" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="C50" t="s">
-        <v>401</v>
+        <v>404</v>
       </c>
       <c r="D50" t="s">
         <v>351</v>
       </c>
       <c r="E50" t="s">
-        <v>255</v>
+        <v>252</v>
       </c>
       <c r="F50">
         <f>SUMIFS('EPS Inputs'!$C$45:$C$99,'EPS Inputs'!$A$45:$A$99,"Hot &amp; Humid",'EPS Inputs'!$D$45:$D$99,$A50)</f>
         <v>0</v>
       </c>
       <c r="G50" s="7">
-        <f>SUMIFS('PNNL Office Measures'!$E$5:$E$69,'PNNL Office Measures'!$A$5:$A$69,$B50,'PNNL Office Measures'!$D$5:$D$69,"Hot &amp; Humid")</f>
-        <v>4019</v>
+        <f>SUMIFS('PNNL Office Measures'!$E$5:$E$69,'PNNL Office Measures'!$A$5:$A$69,$B50,'PNNL Office Measures'!$D$5:$D$69,"Hot &amp; Humid")-$F$32</f>
+        <v>139688</v>
       </c>
       <c r="H50" s="7">
-        <f>SUMIFS('PNNL Office Measures'!$F$5:$F$69,'PNNL Office Measures'!$A$5:$A$69,$B50,'PNNL Office Measures'!$D$5:$D$69,"Hot &amp; Humid")</f>
-        <v>29420</v>
+        <f>SUMIFS('PNNL Office Measures'!$F$5:$F$69,'PNNL Office Measures'!$A$5:$A$69,$B50,'PNNL Office Measures'!$D$5:$D$69,"Hot &amp; Humid")-$G$32</f>
+        <v>73864</v>
       </c>
       <c r="I50">
         <f>SUMIFS('EPS Inputs'!$C$45:$C$99,'EPS Inputs'!$A$45:$A$99,"Hot &amp; Dry",'EPS Inputs'!$D$45:$D$99,$A50)</f>
         <v>0</v>
       </c>
       <c r="J50" s="7">
-        <f>SUMIFS('PNNL Office Measures'!$E$5:$E$69,'PNNL Office Measures'!$A$5:$A$69,$B50,'PNNL Office Measures'!$D$5:$D$69,"Hot &amp; Dry")</f>
-        <v>4635</v>
+        <f>SUMIFS('PNNL Office Measures'!$E$5:$E$69,'PNNL Office Measures'!$A$5:$A$69,$B50,'PNNL Office Measures'!$D$5:$D$69,"Hot &amp; Dry")-$F$33</f>
+        <v>161384</v>
       </c>
       <c r="K50" s="7">
-        <f>SUMIFS('PNNL Office Measures'!$F$5:$F$69,'PNNL Office Measures'!$A$5:$A$69,$B50,'PNNL Office Measures'!$D$5:$D$69,"Hot &amp; Dry")</f>
-        <v>42167</v>
+        <f>SUMIFS('PNNL Office Measures'!$F$5:$F$69,'PNNL Office Measures'!$A$5:$A$69,$B50,'PNNL Office Measures'!$D$5:$D$69,"Hot &amp; Dry")-$G$33</f>
+        <v>74529</v>
       </c>
       <c r="L50">
         <f>SUMIFS('EPS Inputs'!$C$45:$C$99,'EPS Inputs'!$A$45:$A$99,"Marine",'EPS Inputs'!$D$45:$D$99,$A50)</f>
         <v>1</v>
       </c>
       <c r="M50" s="7">
-        <f>SUMIFS('PNNL Office Measures'!$E$5:$E$69,'PNNL Office Measures'!$A$5:$A$69,$B50,'PNNL Office Measures'!$D$5:$D$69,"Marine")</f>
-        <v>5400</v>
+        <f>SUMIFS('PNNL Office Measures'!$E$5:$E$69,'PNNL Office Measures'!$A$5:$A$69,$B50,'PNNL Office Measures'!$D$5:$D$69,"Marine")-$F$34</f>
+        <v>165600</v>
       </c>
       <c r="N50" s="7">
-        <f>SUMIFS('PNNL Office Measures'!$F$5:$F$69,'PNNL Office Measures'!$A$5:$A$69,$B50,'PNNL Office Measures'!$D$5:$D$69,"Marine")</f>
-        <v>38795</v>
+        <f>SUMIFS('PNNL Office Measures'!$F$5:$F$69,'PNNL Office Measures'!$A$5:$A$69,$B50,'PNNL Office Measures'!$D$5:$D$69,"Marine")-$G$34</f>
+        <v>77184</v>
       </c>
       <c r="O50">
         <f>SUMIFS('EPS Inputs'!$C$45:$C$99,'EPS Inputs'!$A$45:$A$99,"Cold",'EPS Inputs'!$D$45:$D$99,$A50)</f>
         <v>1</v>
       </c>
       <c r="P50" s="7">
-        <f>SUMIFS('PNNL Office Measures'!$E$5:$E$69,'PNNL Office Measures'!$A$5:$A$69,$B50,'PNNL Office Measures'!$D$5:$D$69,"Cold")</f>
-        <v>6247</v>
+        <f>SUMIFS('PNNL Office Measures'!$E$5:$E$69,'PNNL Office Measures'!$A$5:$A$69,$B50,'PNNL Office Measures'!$D$5:$D$69,"Cold")-$F$35</f>
+        <v>173248</v>
       </c>
       <c r="Q50" s="7">
-        <f>SUMIFS('PNNL Office Measures'!$F$5:$F$69,'PNNL Office Measures'!$A$5:$A$69,$B50,'PNNL Office Measures'!$D$5:$D$69,"Cold")</f>
-        <v>50985</v>
+        <f>SUMIFS('PNNL Office Measures'!$F$5:$F$69,'PNNL Office Measures'!$A$5:$A$69,$B50,'PNNL Office Measures'!$D$5:$D$69,"Cold")-$G$35</f>
+        <v>73052</v>
       </c>
       <c r="R50">
         <f>SUMIFS('EPS Inputs'!$C$45:$C$99,'EPS Inputs'!$A$45:$A$99,"Very Cold",'EPS Inputs'!$D$45:$D$99,$A50)</f>
         <v>1</v>
       </c>
       <c r="S50" s="7">
-        <f>SUMIFS('PNNL Office Measures'!$E$5:$E$69,'PNNL Office Measures'!$A$5:$A$69,$B50,'PNNL Office Measures'!$D$5:$D$69,"Very Cold")</f>
-        <v>5656</v>
+        <f>SUMIFS('PNNL Office Measures'!$E$5:$E$69,'PNNL Office Measures'!$A$5:$A$69,$B50,'PNNL Office Measures'!$D$5:$D$69,"Very Cold")-$F$36</f>
+        <v>180602</v>
       </c>
       <c r="T50" s="7">
-        <f>SUMIFS('PNNL Office Measures'!$F$5:$F$69,'PNNL Office Measures'!$A$5:$A$69,$B50,'PNNL Office Measures'!$D$5:$D$69,"Very Cold")</f>
-        <v>42463</v>
+        <f>SUMIFS('PNNL Office Measures'!$F$5:$F$69,'PNNL Office Measures'!$A$5:$A$69,$B50,'PNNL Office Measures'!$D$5:$D$69,"Very Cold")-$G$36</f>
+        <v>72757</v>
       </c>
       <c r="U50" s="13">
         <f t="shared" si="0"/>
-        <v>3.2584128844980417E-3</v>
+        <v>0.1151417694856241</v>
       </c>
       <c r="V50" s="13">
         <f t="shared" si="1"/>
-        <v>2.6283874726998013E-2</v>
+        <v>4.8692711496011676E-2</v>
       </c>
       <c r="W50" s="13">
         <f>VLOOKUP($D50,Calcs!$A$21:$J$27,8,FALSE)</f>
@@ -17686,65 +17750,65 @@
       </c>
       <c r="Z50" s="13">
         <f t="shared" si="2"/>
-        <v>1.7730010125589174E-3</v>
+        <v>6.2652119642991694E-2</v>
       </c>
       <c r="AA50" s="13">
         <f t="shared" si="3"/>
-        <v>1.4316634160465903E-3</v>
+        <v>5.0590353302274002E-2</v>
       </c>
       <c r="AB50" s="13">
         <f t="shared" si="4"/>
-        <v>5.3748455892534113E-5</v>
+        <v>1.8992965403584097E-3</v>
       </c>
     </row>
     <row r="51" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A51" s="1" t="s">
-        <v>402</v>
+        <v>405</v>
       </c>
       <c r="G51" s="7">
         <f>SUMPRODUCT(F40:F50,G40:G50)+SUMPRODUCT(F40:F50,H40:H50)</f>
-        <v>857499</v>
+        <v>477093</v>
       </c>
       <c r="J51" s="7">
         <f>SUMPRODUCT(I40:I50,J40:J50)+SUMPRODUCT(I40:I50,K40:K50)</f>
-        <v>1383954</v>
+        <v>1000130</v>
       </c>
       <c r="M51" s="7">
         <f>SUMPRODUCT(L40:L50,M40:M50)+SUMPRODUCT(L40:L50,N40:N50)</f>
-        <v>1217854</v>
+        <v>1018935</v>
       </c>
       <c r="P51" s="7">
         <f>SUMPRODUCT(O40:O50,P40:P50)+SUMPRODUCT(O40:O50,Q40:Q50)</f>
-        <v>1238255</v>
+        <v>1051099</v>
       </c>
       <c r="S51" s="7">
         <f>SUMPRODUCT(R40:R50,S40:S50)+SUMPRODUCT(R40:R50,T40:T50)</f>
-        <v>1225958</v>
+        <v>1056492</v>
       </c>
       <c r="U51" s="13">
         <f>SUM(U40:U50)</f>
-        <v>0.32400416417191263</v>
+        <v>0.39755245056510913</v>
       </c>
       <c r="V51" s="13">
         <f>SUM(V40:V50)</f>
-        <v>0.6759958358280872</v>
+        <v>0.60244754943489109</v>
       </c>
       <c r="Z51" s="13">
         <f>SUM(Z40:Z50)</f>
-        <v>0.26334422640900695</v>
+        <v>0.29027410394788289</v>
       </c>
       <c r="AA51" s="13">
         <f>SUM(AA40:AA50)</f>
-        <v>5.5813720451677588E-2</v>
+        <v>0.10240893888644097</v>
       </c>
       <c r="AB51" s="13">
         <f>SUM(AB40:AB50)</f>
-        <v>4.8462173112280597E-3</v>
+        <v>4.8694077307852874E-3</v>
       </c>
     </row>
     <row r="54" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A54" s="9" t="s">
-        <v>403</v>
+        <v>406</v>
       </c>
       <c r="B54" s="10"/>
       <c r="C54" s="10"/>
@@ -17759,27 +17823,27 @@
     <row r="55" spans="1:28" ht="48" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A55" s="6"/>
       <c r="B55" s="6" t="s">
-        <v>404</v>
+        <v>407</v>
       </c>
       <c r="C55" s="6" t="s">
-        <v>405</v>
+        <v>408</v>
       </c>
       <c r="D55" s="6" t="s">
-        <v>406</v>
+        <v>409</v>
       </c>
       <c r="E55" s="6" t="s">
-        <v>407</v>
+        <v>410</v>
       </c>
       <c r="F55" s="6" t="s">
-        <v>408</v>
+        <v>411</v>
       </c>
       <c r="G55" s="6" t="s">
-        <v>409</v>
+        <v>412</v>
       </c>
     </row>
     <row r="56" spans="1:28" ht="45" x14ac:dyDescent="0.25">
       <c r="A56" s="3" t="s">
-        <v>410</v>
+        <v>413</v>
       </c>
       <c r="B56" s="13">
         <f>INDEX('EPS Inputs'!$B$5:$BA$5,MATCH("ISIC 28",'EPS Inputs'!$B$4:$BA$4,0))</f>
@@ -17798,15 +17862,15 @@
         <v>0.73624568700000004</v>
       </c>
       <c r="F56" t="s">
-        <v>411</v>
+        <v>414</v>
       </c>
       <c r="G56" t="s">
-        <v>411</v>
+        <v>414</v>
       </c>
     </row>
     <row r="57" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A57" s="6" t="s">
-        <v>412</v>
+        <v>415</v>
       </c>
     </row>
     <row r="58" spans="1:28" x14ac:dyDescent="0.25">
@@ -18411,11 +18475,11 @@
       </c>
       <c r="F78" s="16">
         <f t="shared" ref="F78:G97" si="6">SUMIFS($Z$40:$Z$50,$E$40:$E$50,$A78)+IF($A78="ISIC 41T43",$V$51,0)+IF($A78="ISIC 45T47",$AA$51,0)+IF($A78="ISIC 49",$AB$51,0)</f>
-        <v>0</v>
+        <v>6.2652119642991694E-2</v>
       </c>
       <c r="G78" s="16">
         <f t="shared" si="6"/>
-        <v>0</v>
+        <v>6.2652119642991694E-2</v>
       </c>
     </row>
     <row r="79" spans="1:7" x14ac:dyDescent="0.25">
@@ -18440,11 +18504,11 @@
       </c>
       <c r="F79" s="16">
         <f t="shared" si="6"/>
-        <v>0.15189975434567671</v>
+        <v>8.2476824567215584E-2</v>
       </c>
       <c r="G79" s="16">
         <f t="shared" si="6"/>
-        <v>0.15189975434567671</v>
+        <v>8.2476824567215584E-2</v>
       </c>
     </row>
     <row r="80" spans="1:7" x14ac:dyDescent="0.25">
@@ -18469,11 +18533,11 @@
       </c>
       <c r="F80" s="16">
         <f t="shared" si="6"/>
-        <v>2.4713665761134956E-2</v>
+        <v>3.5622900571994909E-2</v>
       </c>
       <c r="G80" s="16">
         <f t="shared" si="6"/>
-        <v>2.4713665761134956E-2</v>
+        <v>3.5622900571994909E-2</v>
       </c>
     </row>
     <row r="81" spans="1:7" x14ac:dyDescent="0.25">
@@ -18498,11 +18562,11 @@
       </c>
       <c r="F81" s="16">
         <f t="shared" si="6"/>
-        <v>6.7850177477708955E-3</v>
+        <v>7.446325552416035E-3</v>
       </c>
       <c r="G81" s="16">
         <f t="shared" si="6"/>
-        <v>6.7850177477708955E-3</v>
+        <v>7.446325552416035E-3</v>
       </c>
     </row>
     <row r="82" spans="1:7" x14ac:dyDescent="0.25">
@@ -18730,11 +18794,11 @@
       </c>
       <c r="F89" s="16">
         <f t="shared" si="6"/>
-        <v>0.75594162438251167</v>
+        <v>0.70452348304815571</v>
       </c>
       <c r="G89" s="16">
         <f t="shared" si="6"/>
-        <v>0.75594162438251167</v>
+        <v>0.70452348304815571</v>
       </c>
     </row>
     <row r="90" spans="1:7" x14ac:dyDescent="0.25">
@@ -18759,11 +18823,11 @@
       </c>
       <c r="F90" s="16">
         <f t="shared" si="6"/>
-        <v>5.5813720451677588E-2</v>
+        <v>0.10240893888644097</v>
       </c>
       <c r="G90" s="16">
         <f t="shared" si="6"/>
-        <v>5.5813720451677588E-2</v>
+        <v>0.10240893888644097</v>
       </c>
     </row>
     <row r="91" spans="1:7" x14ac:dyDescent="0.25">
@@ -18788,11 +18852,11 @@
       </c>
       <c r="F91" s="16">
         <f t="shared" si="6"/>
-        <v>4.8462173112280597E-3</v>
+        <v>4.8694077307852874E-3</v>
       </c>
       <c r="G91" s="16">
         <f t="shared" si="6"/>
-        <v>4.8462173112280597E-3</v>
+        <v>4.8694077307852874E-3</v>
       </c>
     </row>
     <row r="92" spans="1:7" x14ac:dyDescent="0.25">
@@ -19339,11 +19403,11 @@
       </c>
       <c r="F110" s="13">
         <f t="shared" si="8"/>
-        <v>0.99999999999999978</v>
+        <v>1.0000000000000002</v>
       </c>
       <c r="G110" s="13">
         <f t="shared" si="8"/>
-        <v>0.99999999999999978</v>
+        <v>1.0000000000000002</v>
       </c>
     </row>
   </sheetData>
@@ -19368,18 +19432,18 @@
   <sheetData>
     <row r="1" spans="1:3" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="6" t="s">
-        <v>413</v>
+        <v>416</v>
       </c>
       <c r="B1" s="6" t="s">
-        <v>414</v>
+        <v>417</v>
       </c>
       <c r="C1" s="6" t="s">
-        <v>415</v>
+        <v>418</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>416</v>
+        <v>419</v>
       </c>
       <c r="B2">
         <f>SUM('SoBRCbIC-urbanresidential'!B2:BA2)</f>
@@ -19392,7 +19456,7 @@
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>417</v>
+        <v>420</v>
       </c>
       <c r="B3">
         <f>SUM('SoBRCbIC-urbanresidential'!B3:BA3)</f>
@@ -19405,7 +19469,7 @@
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>418</v>
+        <v>421</v>
       </c>
       <c r="B4">
         <f>SUM('SoBRCbIC-urbanresidential'!B4:BA4)</f>
@@ -19418,7 +19482,7 @@
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>419</v>
+        <v>422</v>
       </c>
       <c r="B5">
         <f>SUM('SoBRCbIC-urbanresidential'!B5:BA5)</f>
@@ -19431,7 +19495,7 @@
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>420</v>
+        <v>423</v>
       </c>
       <c r="B6">
         <f>SUM('SoBRCbIC-urbanresidential'!B6:BA6)</f>
@@ -19444,7 +19508,7 @@
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>421</v>
+        <v>424</v>
       </c>
       <c r="B7">
         <f>SUM('SoBRCbIC-urbanresidential'!B7:BA7)</f>
@@ -19457,7 +19521,7 @@
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>422</v>
+        <v>425</v>
       </c>
       <c r="B8">
         <f>SUM('SoBRCbIC-ruralresidential'!B2:BA2)</f>
@@ -19470,7 +19534,7 @@
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>423</v>
+        <v>426</v>
       </c>
       <c r="B9">
         <f>SUM('SoBRCbIC-ruralresidential'!B3:BA3)</f>
@@ -19483,7 +19547,7 @@
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>424</v>
+        <v>427</v>
       </c>
       <c r="B10">
         <f>SUM('SoBRCbIC-ruralresidential'!B4:BA4)</f>
@@ -19496,7 +19560,7 @@
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>425</v>
+        <v>428</v>
       </c>
       <c r="B11">
         <f>SUM('SoBRCbIC-ruralresidential'!B5:BA5)</f>
@@ -19509,7 +19573,7 @@
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>426</v>
+        <v>429</v>
       </c>
       <c r="B12">
         <f>SUM('SoBRCbIC-ruralresidential'!B6:BA6)</f>
@@ -19522,7 +19586,7 @@
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>427</v>
+        <v>430</v>
       </c>
       <c r="B13">
         <f>SUM('SoBRCbIC-ruralresidential'!B7:BA7)</f>
@@ -19535,11 +19599,11 @@
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>428</v>
+        <v>431</v>
       </c>
       <c r="B14">
         <f>SUM('SoBRCbIC-commercial'!B2:BA2)</f>
-        <v>0.99999999999999978</v>
+        <v>1.0000000000000002</v>
       </c>
       <c r="C14">
         <f t="shared" si="0"/>
@@ -19548,11 +19612,11 @@
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>429</v>
+        <v>432</v>
       </c>
       <c r="B15">
         <f>SUM('SoBRCbIC-commercial'!B3:BA3)</f>
-        <v>0.99999999999999978</v>
+        <v>1.0000000000000002</v>
       </c>
       <c r="C15">
         <f t="shared" si="0"/>
@@ -19561,7 +19625,7 @@
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>430</v>
+        <v>433</v>
       </c>
       <c r="B16">
         <f>SUM('SoBRCbIC-commercial'!B4:BA4)</f>
@@ -19574,7 +19638,7 @@
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>431</v>
+        <v>434</v>
       </c>
       <c r="B17">
         <f>SUM('SoBRCbIC-commercial'!B5:BA5)</f>
@@ -19587,7 +19651,7 @@
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>432</v>
+        <v>435</v>
       </c>
       <c r="B18">
         <f>SUM('SoBRCbIC-commercial'!B6:BA6)</f>
@@ -19600,7 +19664,7 @@
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>433</v>
+        <v>436</v>
       </c>
       <c r="B19">
         <f>SUM('SoBRCbIC-commercial'!B7:BA7)</f>
@@ -19613,7 +19677,7 @@
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>434</v>
+        <v>437</v>
       </c>
       <c r="B20">
         <f>INDEX('EPS Inputs'!$B$5:$BA$5,MATCH("ISIC 28",'EPS Inputs'!$B$4:$BA$4,0))+INDEX('EPS Inputs'!$B$5:$BA$5,MATCH("ISIC 41T43",'EPS Inputs'!$B$4:$BA$4,0))</f>
@@ -19626,7 +19690,7 @@
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>435</v>
+        <v>438</v>
       </c>
       <c r="B21">
         <f>INDEX('EPS Inputs'!$B$6:$BA$6,MATCH("ISIC 28",'EPS Inputs'!$B$4:$BA$4,0))+INDEX('EPS Inputs'!$B$6:$BA$6,MATCH("ISIC 41T43",'EPS Inputs'!$B$4:$BA$4,0))</f>
@@ -19639,7 +19703,7 @@
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>436</v>
+        <v>439</v>
       </c>
       <c r="B22">
         <f>INDEX('EPS Inputs'!$B$14:$BA$14,MATCH("ISIC 28",'EPS Inputs'!$B$13:$BA$13,0))+INDEX('EPS Inputs'!$B$14:$BA$14,MATCH("ISIC 41T43",'EPS Inputs'!$B$13:$BA$13,0))</f>
@@ -19652,7 +19716,7 @@
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>437</v>
+        <v>440</v>
       </c>
       <c r="B23">
         <f>INDEX('EPS Inputs'!$B$15:$BA$15,MATCH("ISIC 28",'EPS Inputs'!$B$13:$BA$13,0))+INDEX('EPS Inputs'!$B$15:$BA$15,MATCH("ISIC 41T43",'EPS Inputs'!$B$13:$BA$13,0))</f>
@@ -19665,11 +19729,11 @@
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>438</v>
+        <v>441</v>
       </c>
       <c r="B24">
         <f>Calcs!U51+Calcs!V51</f>
-        <v>0.99999999999999978</v>
+        <v>1.0000000000000002</v>
       </c>
       <c r="C24">
         <f t="shared" si="1"/>
@@ -19678,7 +19742,7 @@
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>439</v>
+        <v>442</v>
       </c>
       <c r="B25">
         <f>SUM(Calcs!D32:D36)</f>
@@ -19691,7 +19755,7 @@
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>440</v>
+        <v>443</v>
       </c>
       <c r="B26">
         <f>Calcs!B16</f>
@@ -19704,7 +19768,7 @@
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>441</v>
+        <v>444</v>
       </c>
       <c r="B27">
         <f>Calcs!H21+Calcs!I21+Calcs!J21</f>
@@ -19717,7 +19781,7 @@
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>442</v>
+        <v>445</v>
       </c>
       <c r="B28">
         <f>Calcs!H22+Calcs!I22+Calcs!J22</f>
@@ -19730,7 +19794,7 @@
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>443</v>
+        <v>446</v>
       </c>
       <c r="B29">
         <f>Calcs!H23+Calcs!I23+Calcs!J23</f>
@@ -19743,7 +19807,7 @@
     </row>
     <row r="30" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>444</v>
+        <v>447</v>
       </c>
       <c r="B30">
         <f>Calcs!H24+Calcs!I24+Calcs!J24</f>
@@ -19756,7 +19820,7 @@
     </row>
     <row r="31" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>445</v>
+        <v>448</v>
       </c>
       <c r="B31">
         <f>Calcs!H25+Calcs!I25+Calcs!J25</f>
@@ -19769,7 +19833,7 @@
     </row>
     <row r="33" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A33" s="1" t="s">
-        <v>446</v>
+        <v>449</v>
       </c>
       <c r="C33" s="1">
         <f>SUM(C2:C31)</f>

</xml_diff>